<commit_message>
Updated scripts so that delivery rate, latency and false negative calculations can be done all at once
</commit_message>
<xml_diff>
--- a/data/Experiment1Data.xlsx
+++ b/data/Experiment1Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jon/USRA2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4856D360-A793-6943-A1C7-ED56EAF49AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC845E2-989F-1A4F-9251-D511C5E7CB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13380" yWindow="500" windowWidth="15420" windowHeight="17460" activeTab="1" xr2:uid="{348090C3-978A-6043-9FDD-83C972258579}"/>
+    <workbookView xWindow="3760" yWindow="500" windowWidth="19080" windowHeight="17460" activeTab="1" xr2:uid="{348090C3-978A-6043-9FDD-83C972258579}"/>
   </bookViews>
   <sheets>
     <sheet name="500m Commons Test" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="34">
   <si>
     <t>SHORT_TURBO</t>
   </si>
@@ -124,6 +124,21 @@
   </si>
   <si>
     <t>Actual (RSSI - dBm)</t>
+  </si>
+  <si>
+    <t>Test: Max distance within city</t>
+  </si>
+  <si>
+    <t>Hypothesized (m)</t>
+  </si>
+  <si>
+    <t>Actual (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">725m (uphill), </t>
+  </si>
+  <si>
+    <t>Down+A12</t>
   </si>
 </sst>
 </file>
@@ -172,11 +187,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -859,9 +875,275 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7173A505-736B-0B42-8513-F335C17B4FD4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="19.5" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2">
+        <v>-117</v>
+      </c>
+      <c r="E2">
+        <v>0.3</v>
+      </c>
+      <c r="F2">
+        <v>21.88</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2">
+        <v>500</v>
+      </c>
+      <c r="J2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>-121</v>
+      </c>
+      <c r="E3">
+        <v>0.2</v>
+      </c>
+      <c r="F3">
+        <v>10.94</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3">
+        <v>250</v>
+      </c>
+      <c r="J3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>-124</v>
+      </c>
+      <c r="E4">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="F4">
+        <v>6.25</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4">
+        <v>250</v>
+      </c>
+      <c r="J4">
+        <v>145.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>-127</v>
+      </c>
+      <c r="E5">
+        <v>0.1</v>
+      </c>
+      <c r="F5">
+        <v>3.52</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5">
+        <v>250</v>
+      </c>
+      <c r="J5">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>-130</v>
+      </c>
+      <c r="E6">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F6">
+        <v>1.95</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6">
+        <v>250</v>
+      </c>
+      <c r="J6">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>-133</v>
+      </c>
+      <c r="E7">
+        <v>0.05</v>
+      </c>
+      <c r="F7">
+        <v>1.07</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7">
+        <v>250</v>
+      </c>
+      <c r="J7">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8">
+        <v>-136</v>
+      </c>
+      <c r="E8">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="F8">
+        <v>0.34</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8">
+        <v>125</v>
+      </c>
+      <c r="J8">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>-137</v>
+      </c>
+      <c r="E9">
+        <v>3.15E-2</v>
+      </c>
+      <c r="F9">
+        <v>0.18</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9">
+        <v>125</v>
+      </c>
+      <c r="J9">
+        <v>158.80000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>